<commit_message>
New dashboard + finish off updated bank worksheet design to 18 (or 19) sheet spreadsheets
Untracks 6 regenerated research/ derived-data artifacts that grew past
GitHub's 100MB file limit (insights.db, bank_metrics.csv, in017/in023/
in025 JSON payloads, powerbi/fact_observation.csv) and adds them to
.gitignore. They stay on disk and rebuild via
`python3 scripts/insights/refresh_all.py`; only the regenerable size, not
the underlying source data, made them too large to track in git.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lm3sZFNN1p9FpS4j3VgT3X
</commit_message>
<xml_diff>
--- a/banks/AFIN BANK FINANCIALS.xlsx
+++ b/banks/AFIN BANK FINANCIALS.xlsx
@@ -8,18 +8,23 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow Statement" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CET1 Capital" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CET1 Ratio" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 1 Capital" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 1 Ratio" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Capital" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Capital Ratio" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total RWAs" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leverage Ratio" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LCR" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NSFR" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MREL Ratio" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profit &amp; Loss" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statement of Changes in Equity" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow Statement" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset Quality" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CET1 Capital" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CET1 Ratio" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 1 Capital" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 1 Ratio" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Capital" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Capital Ratio" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total RWAs" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RWA Breakdown" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leverage Ratio" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LCR" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NSFR" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MREL Ratio" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -203,7 +208,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Afin Bank Limited — Cash Flow Summary by Year</a:t>
+              <a:t>Afin Bank Limited — Balance Sheet Summary by Year</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -298,30 +303,6 @@
             </numRef>
           </val>
         </ser>
-        <ser>
-          <idx val="3"/>
-          <order val="3"/>
-          <tx>
-            <strRef>
-              <f>'Overview'!E9</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Overview'!$F$5</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Overview'!$F$9</f>
-            </numRef>
-          </val>
-        </ser>
         <gapWidth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
@@ -401,6 +382,552 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:t>Afin Bank Limited — Profit &amp; Loss Summary by Year</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <layout>
+        <manualLayout>
+          <layoutTarget val="inner"/>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.1"/>
+          <y val="0.14"/>
+          <w val="0.85"/>
+          <h val="0.55"/>
+        </manualLayout>
+      </layout>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!I12</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Overview'!$J$11</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$J$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!I13</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Overview'!$J$11</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$J$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="b"/>
+        <majorTickMark val="out"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>£</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="out"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+      <layout>
+        <manualLayout>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.02"/>
+          <y val="0.84"/>
+          <w val="0.96"/>
+          <h val="0.16"/>
+        </manualLayout>
+      </layout>
+    </legend>
+    <plotVisOnly val="0"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Afin Bank Limited — Statement of Changes in Equity Summary by Year</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <layout>
+        <manualLayout>
+          <layoutTarget val="inner"/>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.1"/>
+          <y val="0.14"/>
+          <w val="0.85"/>
+          <h val="0.55"/>
+        </manualLayout>
+      </layout>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!M17</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Overview'!$N$16</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$N$17</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!M18</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Overview'!$N$16</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$N$18</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!M19</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Overview'!$N$16</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$N$19</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!M20</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Overview'!$N$16</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$N$20</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="b"/>
+        <majorTickMark val="out"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>£</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="out"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+      <layout>
+        <manualLayout>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.02"/>
+          <y val="0.84"/>
+          <w val="0.96"/>
+          <h val="0.16"/>
+        </manualLayout>
+      </layout>
+    </legend>
+    <plotVisOnly val="0"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Afin Bank Limited — Cash Flow Summary by Year</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <layout>
+        <manualLayout>
+          <layoutTarget val="inner"/>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.1"/>
+          <y val="0.14"/>
+          <w val="0.85"/>
+          <h val="0.55"/>
+        </manualLayout>
+      </layout>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!Q24</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Overview'!$R$23</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$R$24</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!Q25</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Overview'!$R$23</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$R$25</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!Q26</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Overview'!$R$23</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$R$26</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!Q27</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Overview'!$R$23</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$R$27</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="b"/>
+        <majorTickMark val="out"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>£</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="out"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+      <layout>
+        <manualLayout>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.02"/>
+          <y val="0.84"/>
+          <w val="0.96"/>
+          <h val="0.16"/>
+        </manualLayout>
+      </layout>
+    </legend>
+    <plotVisOnly val="0"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
               <a:t>Afin Bank Limited — Pillar 3 Key Metrics by Year</a:t>
             </a:r>
           </a:p>
@@ -428,7 +955,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Overview'!I6</f>
+              <f>'Overview'!U6</f>
             </strRef>
           </tx>
           <spPr>
@@ -446,12 +973,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$J$5</f>
+              <f>'Overview'!$V$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$J$6</f>
+              <f>'Overview'!$V$6</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -461,7 +988,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Overview'!I7</f>
+              <f>'Overview'!U7</f>
             </strRef>
           </tx>
           <spPr>
@@ -479,12 +1006,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$J$5</f>
+              <f>'Overview'!$V$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$J$7</f>
+              <f>'Overview'!$V$7</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -494,7 +1021,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Overview'!I8</f>
+              <f>'Overview'!U8</f>
             </strRef>
           </tx>
           <spPr>
@@ -512,12 +1039,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$J$5</f>
+              <f>'Overview'!$V$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$J$8</f>
+              <f>'Overview'!$V$8</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -527,7 +1054,7 @@
           <order val="3"/>
           <tx>
             <strRef>
-              <f>'Overview'!I9</f>
+              <f>'Overview'!U9</f>
             </strRef>
           </tx>
           <spPr>
@@ -545,12 +1072,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$J$5</f>
+              <f>'Overview'!$V$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$J$9</f>
+              <f>'Overview'!$V$9</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -560,7 +1087,7 @@
           <order val="4"/>
           <tx>
             <strRef>
-              <f>'Overview'!I10</f>
+              <f>'Overview'!U10</f>
             </strRef>
           </tx>
           <spPr>
@@ -578,12 +1105,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$J$5</f>
+              <f>'Overview'!$V$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$J$10</f>
+              <f>'Overview'!$V$10</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -593,7 +1120,7 @@
           <order val="5"/>
           <tx>
             <strRef>
-              <f>'Overview'!I11</f>
+              <f>'Overview'!U11</f>
             </strRef>
           </tx>
           <spPr>
@@ -611,12 +1138,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$J$5</f>
+              <f>'Overview'!$V$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$J$11</f>
+              <f>'Overview'!$V$11</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -693,7 +1220,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>22</row>
+      <row>40</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="4680000"/>
@@ -715,10 +1242,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>44</row>
+      <row>62</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8640000" cy="5760000"/>
+    <ext cx="8640000" cy="4680000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -728,6 +1255,72 @@
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>84</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8640000" cy="4680000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>106</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8640000" cy="4680000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>128</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8640000" cy="5760000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="5" name="Chart 5"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1025,7 +1618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:V38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1036,6 +1629,18 @@
     <col hidden="1" width="13" customWidth="1" min="8" max="8"/>
     <col hidden="1" width="13" customWidth="1" min="9" max="9"/>
     <col hidden="1" width="13" customWidth="1" min="10" max="10"/>
+    <col hidden="1" width="13" customWidth="1" min="11" max="11"/>
+    <col hidden="1" width="13" customWidth="1" min="12" max="12"/>
+    <col hidden="1" width="13" customWidth="1" min="13" max="13"/>
+    <col hidden="1" width="13" customWidth="1" min="14" max="14"/>
+    <col hidden="1" width="13" customWidth="1" min="15" max="15"/>
+    <col hidden="1" width="13" customWidth="1" min="16" max="16"/>
+    <col hidden="1" width="13" customWidth="1" min="17" max="17"/>
+    <col hidden="1" width="13" customWidth="1" min="18" max="18"/>
+    <col hidden="1" width="13" customWidth="1" min="19" max="19"/>
+    <col hidden="1" width="13" customWidth="1" min="20" max="20"/>
+    <col hidden="1" width="13" customWidth="1" min="21" max="21"/>
+    <col hidden="1" width="13" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1048,14 +1653,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Summary of cash flow and Pillar 3 disclosures across all years covered in this workbook</t>
+          <t>Headline balance sheet, profit &amp; loss, cash flow and Pillar 3 figures across all years covered in this workbook - how the bank is using its money and the risk it is taking with it</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Cash Flow Summary (£)</t>
+          <t>Balance Sheet Summary (£)</t>
         </is>
       </c>
     </row>
@@ -1075,7 +1680,7 @@
           <t>FY2024</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>FY2024</t>
         </is>
@@ -1084,226 +1689,460 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Net cash outflow from operating activities</t>
+          <t>Total assets</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-5854403</v>
+        <v>17427943</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Net cash outflow from operating activities</t>
+          <t>Total assets</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>-5854403</v>
-      </c>
-      <c r="I6" t="inlineStr">
+        <v>17427943</v>
+      </c>
+      <c r="U6" t="inlineStr">
         <is>
           <t>CET1 Ratio</t>
         </is>
       </c>
-      <c r="J6" t="n">
+      <c r="V6" t="n">
         <v>418.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Net cash used in investing activities</t>
+          <t>Trade and other payables</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>-12345649</v>
+        <v>1102894</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Net cash used in investing activities</t>
+          <t>Trade and other payables</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>-12345649</v>
-      </c>
-      <c r="I7" t="inlineStr">
+        <v>1102894</v>
+      </c>
+      <c r="U7" t="inlineStr">
         <is>
           <t>Tier 1 Ratio</t>
         </is>
       </c>
-      <c r="J7" t="n">
+      <c r="V7" t="n">
         <v>418.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
+          <t>Total equity</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>15359865</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Total equity</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>15359865</v>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Total Capital Ratio</t>
+        </is>
+      </c>
+      <c r="V8" t="n">
+        <v>418.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Leverage Ratio</t>
+        </is>
+      </c>
+      <c r="V9" t="n">
+        <v>87.40000000000001</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Profit &amp; Loss Summary (£)</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>LCR</t>
+        </is>
+      </c>
+      <c r="V10" t="n">
+        <v>999999</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Line item</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>NSFR</t>
+        </is>
+      </c>
+      <c r="V11" t="n">
+        <v>492.2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Total operating expenses</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>-6256733</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Total operating expenses</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>-6256733</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Loss for the year</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>-6193551</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Loss for the year</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>-6193551</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Statement of Changes in Equity Summary (£)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Line item</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Opening equity</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>962179</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Opening equity</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>962179</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Total comprehensive income</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>-6126169</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Total comprehensive income</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>-6126169</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Other movements, net</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>20523855</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Other movements, net</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>20523855</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Closing equity</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>15359865</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Closing equity</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>15359865</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Cash Flow Summary (£)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Line item</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Net cash outflow from operating activities</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>-5854403</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Net cash outflow from operating activities</t>
+        </is>
+      </c>
+      <c r="R24" t="n">
+        <v>-5854403</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Net cash used in investing activities</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>-12345649</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Net cash used in investing activities</t>
+        </is>
+      </c>
+      <c r="R25" t="n">
+        <v>-12345649</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
           <t>Net cash generated from financing activities</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B26" s="5" t="n">
         <v>20384295</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="Q26" t="inlineStr">
         <is>
           <t>Net cash generated from financing activities</t>
         </is>
       </c>
-      <c r="F8" t="n">
+      <c r="R26" t="n">
         <v>20384295</v>
       </c>
-      <c r="I8" t="inlineStr">
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at end of year</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>3155921</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at end of year</t>
+        </is>
+      </c>
+      <c r="R27" t="n">
+        <v>3155921</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Pillar 3 Key Metrics</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Line item</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>CET1 Ratio</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>418.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Tier 1 Ratio</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>418.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>Total Capital Ratio</t>
         </is>
       </c>
-      <c r="J8" t="n">
-        <v>418.5</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Cash and cash equivalents at end of year</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>3155921</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Cash and cash equivalents at end of year</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>3155921</v>
-      </c>
-      <c r="I9" t="inlineStr">
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>418.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>Leverage Ratio</t>
         </is>
       </c>
-      <c r="J9" t="n">
-        <v>87.40000000000001</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="I10" t="inlineStr">
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>87.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>LCR</t>
         </is>
       </c>
-      <c r="J10" t="n">
-        <v>999999</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Pillar 3 Key Metrics</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>999999%</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>NSFR</t>
         </is>
       </c>
-      <c r="J11" t="n">
-        <v>492.2</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Line item</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>FY2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>CET1 Ratio</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>418.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Tier 1 Ratio</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>418.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Total Capital Ratio</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>418.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Leverage Ratio</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>87.4%</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>LCR</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>999999%</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>NSFR</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>492.2%</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="45" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>Note: SHORT PERIOD: This workbook intentionally covers FY2024 only. Afin's first Pillar 3 report states that it was authorised as a bank with restrictions in October 2024 and does not provide prior-period comparatives. The Pillar 3 metrics are standalone Afin Bank Limited disclosures; the cash-flow statement is from the audited annual accounts. See each detail sheet for the source citation.</t>
+    <row r="38" ht="45" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>Note: SHORT PERIOD: This workbook intentionally covers FY2024 only. Afin's first Pillar 3 report states that it was authorised as a bank with restrictions in October 2024 and does not provide prior-period comparatives. The Pillar 3 metrics are standalone Afin Bank Limited disclosures; the cash-flow statement is from the audited annual accounts. See each detail sheet for the source citation. Asset Quality and RWA Breakdown are marked not publicly disclosed: Afin has no lending product on its balance sheet yet and, as a small non-complex institution, its Pillar 3 report has no exposure-class RWA table.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A38:B38"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1311,6 +2150,347 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="56" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Afin Bank Limited — Tier 1 Ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>% of RWA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Tier 1 ratio</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>418.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="145" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
+FY2024: UK KM1 Key Metrics, printed pp. 4-5, and UK OV1, printed p. 5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
+Afin Bank annual reports and disclosures page - https://afinbank.com/about/annual-reports-and-disclosures/
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A6:B6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="56" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Afin Bank Limited — Total Capital</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>£'000</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Total capital</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>12922</v>
+      </c>
+    </row>
+    <row r="6" ht="145" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
+FY2024: UK KM1 Key Metrics, printed pp. 4-5, and UK OV1, printed p. 5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
+Afin Bank annual reports and disclosures page - https://afinbank.com/about/annual-reports-and-disclosures/
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A6:B6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="56" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Afin Bank Limited — Total Capital Ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>% of RWA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Total capital ratio</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>418.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="145" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
+FY2024: UK KM1 Key Metrics, printed pp. 4-5, and UK OV1, printed p. 5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
+Afin Bank annual reports and disclosures page - https://afinbank.com/about/annual-reports-and-disclosures/
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A6:B6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="56" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Afin Bank Limited — Total RWAs</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>£'000</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Total risk-weighted exposure amount</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>3087</v>
+      </c>
+    </row>
+    <row r="6" ht="145" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
+FY2024: UK KM1 Key Metrics, printed pp. 4-5, and UK OV1, printed p. 5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
+Afin Bank annual reports and disclosures page - https://afinbank.com/about/annual-reports-and-disclosures/
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A6:B6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Afin Bank Limited — RWA Breakdown</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Afin Bank Limited risk-weighted exposure amount breakdown; amounts in £'000.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Line item</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>FY2024 (£'000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Not publicly disclosed</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Not publicly disclosed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="150" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
+UK KM1 Key Metrics, printed pp. 4-5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.
+NOT DISCLOSED: as a small non-complex institution under CRR Article 433b, Afin Bank's 2024 Pillar 3 disclosure contains only the single aggregate Total RWA figure in UK KM1 (see the Total RWAs sheet) - no UK OV1 exposure-class breakdown is published.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A6:B6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1389,7 +2569,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1506,7 +2686,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1595,7 +2775,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1674,24 +2854,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Afin Bank Limited — Cash Flow Statement</t>
+          <t>Afin Bank Limited — Consolidated Statement of Financial Position</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Afin Bank Limited audited standalone statement of cash flows; amounts in £.</t>
+          <t>Afin Bank Limited audited statement of financial position; amounts in £.</t>
         </is>
       </c>
     </row>
@@ -1710,7 +2890,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Cash flows from operating activities</t>
+          <t>Assets</t>
         </is>
       </c>
       <c r="B4" s="6" t="n"/>
@@ -1718,85 +2898,87 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Cash absorbed by operations</t>
+          <t>Cash and cash equivalents</t>
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>-5854403</v>
+        <v>3155921</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Net cash outflow from operating activities</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n">
-        <v>-5854403</v>
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Treasury assets</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>9767797</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Investing activities</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n"/>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Receivables</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>450628</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Purchase of intangible assets</t>
+          <t>Prepayments</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>-2668378</v>
+        <v>372022</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Purchase of property, plant and equipment</t>
+          <t>Property, plant and equipment</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>-52008</v>
+        <v>57172</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Purchase of investments</t>
+          <t>Right-of-use assets</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>-9700415</v>
+        <v>967204</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Finance income</t>
+          <t>Intangible assets</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>75152</v>
+        <v>2657199</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Net cash used in investing activities</t>
+          <t>Total assets</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>-12345649</v>
+        <v>17427943</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Financing activities</t>
+          <t>Liabilities</t>
         </is>
       </c>
       <c r="B13" s="6" t="n"/>
@@ -1804,87 +2986,114 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Proceeds from issue of shares</t>
+          <t>Trade and other payables</t>
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>20523855</v>
+        <v>1102894</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Payment of lease liabilities</t>
+          <t>Lease liabilities</t>
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>-134783</v>
+        <v>965184</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Finance cost</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="n">
-        <v>-4777</v>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Total liabilities</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>2068078</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Net cash generated from financing activities</t>
+          <t>Net assets</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>20384295</v>
+        <v>15359865</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Net increase in cash and cash equivalents</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="n">
-        <v>2184243</v>
-      </c>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Cash and cash equivalents at the beginning of the year</t>
+          <t>Called up share capital</t>
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>971678</v>
+        <v>23614036</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Cash and cash equivalents at the end of the year</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="n">
-        <v>3155921</v>
-      </c>
-    </row>
-    <row r="22" ht="165" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Revaluation reserve</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n">
+        <v>67382</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Share based payment reserve</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n">
+        <v>267626</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Retained earnings</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n">
+        <v>-8589179</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Total equity</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>15359865</v>
+      </c>
+    </row>
+    <row r="25" ht="150" customHeight="1">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>Sources - Afin Bank Limited audited annual report and financial statements for the year ended 31 December 2024:
-FY2024: Statement of cash flows, printed p. 36 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-Ltd-Year-End-Accounts-FV24-FINAL-SIGNED.pdf
-Companies House 2024 accounts filing (filed 29 September 2025) - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history/MzQ4MjgwOTc2M2FkaXF6a2N4/document?download=0&amp;format=pdf
-Companies House filing history - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
+FY2024: Statement of financial position, printed p. 34 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-Ltd-Year-End-Accounts-FV24-FINAL-SIGNED.pdf
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.
+PRESENTATION NOTE: The source statement also shows FY2023 comparatives on its face, but this workbook is intentionally FY2024-only for consistency with the Cash Flow Statement and Pillar 3 sheets, whose primary source (the 2024 Pillar 3 report) explicitly states no prior-period comparatives are provided.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A25:B25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1896,62 +3105,208 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="56" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Afin Bank Limited — CET1 Capital</t>
+          <t>Afin Bank Limited — Consolidated Statement of Comprehensive Income</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>£'000</t>
+          <t>Afin Bank Limited audited statement of comprehensive income; amounts in £.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Metric</t>
+          <t>Line item</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>FY2024</t>
+          <t>FY2024 (£)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Common Equity Tier 1 (CET1) capital</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="n">
-        <v>12922</v>
-      </c>
-    </row>
-    <row r="6" ht="145" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
-FY2024: UK KM1 Key Metrics, printed pp. 4-5, and UK OV1, printed p. 5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
-Afin Bank annual reports and disclosures page - https://afinbank.com/about/annual-reports-and-disclosures/
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Operating expenses</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Staff costs</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>-3941455</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Depreciation</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>-142504</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Amortisation of intangibles</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>-23179</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Other operating costs</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>-2149595</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Total operating expenses</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>-6256733</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Operating loss</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>-6256733</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Finance income</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>75152</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Finance costs</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>-11970</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Loss before taxation</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>-6193551</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Income tax expense</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Loss for the year</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>-6193551</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Other comprehensive income</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Treasury asset revaluation</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>67382</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Total other comprehensive income for the year</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>67382</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Total comprehensive income for the year</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>-6126169</v>
+      </c>
+    </row>
+    <row r="21" ht="150" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Sources - Afin Bank Limited audited annual report and financial statements for the year ended 31 December 2024:
+FY2024: Statement of comprehensive income, printed p. 33 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-Ltd-Year-End-Accounts-FV24-FINAL-SIGNED.pdf
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.
+PRESENTATION NOTE: The source statement also shows FY2023 comparatives on its face, but this workbook is intentionally FY2024-only for consistency with the Cash Flow Statement and Pillar 3 sheets.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A21:B21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1963,64 +3318,252 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="56" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Afin Bank Limited — CET1 Ratio</t>
+          <t>Afin Bank Limited — Statement of Changes in Equity</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>% of RWA</t>
+          <t>Afin Bank Limited audited statement of changes in equity, 1 January 2023 to 31 December 2024; amounts in £.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Metric</t>
+          <t>Movement</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>FY2024</t>
+          <t>Share capital</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Revaluation reserve</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Share based payment</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Retained earnings</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Total equity</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Common Equity Tier 1 (CET1) ratio</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>418.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="145" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
-FY2024: UK KM1 Key Metrics, printed pp. 4-5, and UK OV1, printed p. 5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
-Afin Bank annual reports and disclosures page - https://afinbank.com/about/annual-reports-and-disclosures/
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Balance at 1 January 2023</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>590654</v>
+      </c>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n">
+        <v>-626440</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>-35786</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Total comprehensive income for the year (2023)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n">
+        <v>-1769188</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>-1769188</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Issue of share capital (2023)</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>2767153</v>
+      </c>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n">
+        <v>2767153</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Balance at 31 December 2023</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>3357807</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>-2395628</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>962179</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Loss for the year (2024)</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n">
+        <v>-6193551</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>-6193551</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Other comprehensive income - Treasury asset revaluation (2024)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n">
+        <v>67382</v>
+      </c>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n">
+        <v>67382</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Total comprehensive income for the year (2024)</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n">
+        <v>67382</v>
+      </c>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n">
+        <v>-6193551</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>-6126169</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Issue of share capital (2024)</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>20256229</v>
+      </c>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n">
+        <v>20256229</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Share based payment (2024)</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n">
+        <v>267626</v>
+      </c>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n">
+        <v>267626</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Balance at 31 December 2024</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>23614036</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>67382</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>267626</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>-8589179</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>15359865</v>
+      </c>
+    </row>
+    <row r="15" ht="150" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Sources - Afin Bank Limited audited annual report and financial statements for the year ended 31 December 2024:
+Statement of changes in equity, printed p. 35, covering 1 January 2023 to 31 December 2024 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-Ltd-Year-End-Accounts-FV24-FINAL-SIGNED.pdf
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.
+This is the one sheet in the workbook that includes FY2023 movements, since the equity roll-forward is chronological (not year-columned) and both years' movements are disclosed on the statement's face.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2032,62 +3575,217 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="56" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Afin Bank Limited — Tier 1 Capital</t>
+          <t>Afin Bank Limited — Cash Flow Statement</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>£'000</t>
+          <t>Afin Bank Limited audited standalone statement of cash flows; amounts in £.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Metric</t>
+          <t>Line item</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>FY2024</t>
+          <t>FY2024 (£)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Tier 1 capital</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="n">
-        <v>12922</v>
-      </c>
-    </row>
-    <row r="6" ht="145" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
-FY2024: UK KM1 Key Metrics, printed pp. 4-5, and UK OV1, printed p. 5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
-Afin Bank annual reports and disclosures page - https://afinbank.com/about/annual-reports-and-disclosures/
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Cash flows from operating activities</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Cash absorbed by operations</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>-5854403</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Net cash outflow from operating activities</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>-5854403</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Investing activities</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Purchase of intangible assets</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>-2668378</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Purchase of property, plant and equipment</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>-52008</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Purchase of investments</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>-9700415</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Finance income</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>75152</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Net cash used in investing activities</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>-12345649</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Financing activities</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Proceeds from issue of shares</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>20523855</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Payment of lease liabilities</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>-134783</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Finance cost</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>-4777</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Net cash generated from financing activities</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>20384295</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Net increase in cash and cash equivalents</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>2184243</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at the beginning of the year</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>971678</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at the end of the year</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>3155921</v>
+      </c>
+    </row>
+    <row r="22" ht="165" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Sources - Afin Bank Limited audited annual report and financial statements for the year ended 31 December 2024:
+FY2024: Statement of cash flows, printed p. 36 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-Ltd-Year-End-Accounts-FV24-FINAL-SIGNED.pdf
+Companies House 2024 accounts filing (filed 29 September 2025) - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history/MzQ4MjgwOTc2M2FkaXF6a2N4/document?download=0&amp;format=pdf
+Companies House filing history - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history
 ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A22:B22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2102,55 +3800,56 @@
   <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="56" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Afin Bank Limited — Tier 1 Ratio</t>
+          <t>Afin Bank Limited — Asset Quality / Credit Risk Disclosures</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>% of RWA</t>
+          <t>Afin Bank Limited loan book / credit risk disclosures; amounts in £.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Metric</t>
+          <t>Line item</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>FY2024</t>
+          <t>FY2024 (£)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Tier 1 ratio</t>
+          <t>Not publicly disclosed</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>418.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="145" customHeight="1">
+          <t>Not publicly disclosed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="150" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
-FY2024: UK KM1 Key Metrics, printed pp. 4-5, and UK OV1, printed p. 5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
-Afin Bank annual reports and disclosures page - https://afinbank.com/about/annual-reports-and-disclosures/
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
+          <t>Sources - Afin Bank Limited 2024 Annual Report and Pillar 3 Disclosures:
+https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-Ltd-Year-End-Accounts-FV24-FINAL-SIGNED.pdf
+https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.
+NOT DISCLOSED: Afin Bank's balance sheet has no lending product line (assets are Cash, Treasury assets, Receivables, Prepayments, PP&amp;E and intangibles only) and neither the 2024 Annual Report nor the 2024 Pillar 3 disclosure (a small non-complex institution under CRR Article 433b) contains a loan book / IFRS 9 stage / credit risk exposure breakdown.</t>
         </is>
       </c>
     </row>
@@ -2178,7 +3877,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Afin Bank Limited — Total Capital</t>
+          <t>Afin Bank Limited — CET1 Capital</t>
         </is>
       </c>
     </row>
@@ -2204,7 +3903,7 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Total capital</t>
+          <t>Common Equity Tier 1 (CET1) capital</t>
         </is>
       </c>
       <c r="B4" s="6" t="n">
@@ -2245,7 +3944,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Afin Bank Limited — Total Capital Ratio</t>
+          <t>Afin Bank Limited — CET1 Ratio</t>
         </is>
       </c>
     </row>
@@ -2271,7 +3970,7 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Total capital ratio</t>
+          <t>Common Equity Tier 1 (CET1) ratio</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -2314,7 +4013,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Afin Bank Limited — Total RWAs</t>
+          <t>Afin Bank Limited — Tier 1 Capital</t>
         </is>
       </c>
     </row>
@@ -2340,11 +4039,11 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Total risk-weighted exposure amount</t>
+          <t>Tier 1 capital</t>
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>3087</v>
+        <v>12922</v>
       </c>
     </row>
     <row r="6" ht="145" customHeight="1">

</xml_diff>

<commit_message>
forgot to commit, finished addition of historical data + audit all banks
</commit_message>
<xml_diff>
--- a/banks/AFIN BANK FINANCIALS.xlsx
+++ b/banks/AFIN BANK FINANCIALS.xlsx
@@ -236,7 +236,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Overview'!E6</f>
+              <f>'Overview'!H6</f>
             </strRef>
           </tx>
           <spPr>
@@ -246,12 +246,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overview'!$F$5</f>
+              <f>'Overview'!$I$5:$L$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$F$6</f>
+              <f>'Overview'!$I$6:$L$6</f>
             </numRef>
           </val>
         </ser>
@@ -260,7 +260,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Overview'!E7</f>
+              <f>'Overview'!H7</f>
             </strRef>
           </tx>
           <spPr>
@@ -270,12 +270,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overview'!$F$5</f>
+              <f>'Overview'!$I$5:$L$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$F$7</f>
+              <f>'Overview'!$I$7:$L$7</f>
             </numRef>
           </val>
         </ser>
@@ -284,7 +284,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Overview'!E8</f>
+              <f>'Overview'!H8</f>
             </strRef>
           </tx>
           <spPr>
@@ -294,12 +294,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overview'!$F$5</f>
+              <f>'Overview'!$I$5:$L$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$F$8</f>
+              <f>'Overview'!$I$8:$L$8</f>
             </numRef>
           </val>
         </ser>
@@ -410,7 +410,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Overview'!I12</f>
+              <f>'Overview'!O12</f>
             </strRef>
           </tx>
           <spPr>
@@ -420,12 +420,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overview'!$J$11</f>
+              <f>'Overview'!$P$11:$S$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$J$12</f>
+              <f>'Overview'!$P$12:$S$12</f>
             </numRef>
           </val>
         </ser>
@@ -434,7 +434,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Overview'!I13</f>
+              <f>'Overview'!O13</f>
             </strRef>
           </tx>
           <spPr>
@@ -444,12 +444,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overview'!$J$11</f>
+              <f>'Overview'!$P$11:$S$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$J$13</f>
+              <f>'Overview'!$P$13:$S$13</f>
             </numRef>
           </val>
         </ser>
@@ -560,7 +560,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Overview'!M17</f>
+              <f>'Overview'!V17</f>
             </strRef>
           </tx>
           <spPr>
@@ -570,12 +570,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overview'!$N$16</f>
+              <f>'Overview'!$W$16:$Z$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$N$17</f>
+              <f>'Overview'!$W$17:$Z$17</f>
             </numRef>
           </val>
         </ser>
@@ -584,7 +584,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Overview'!M18</f>
+              <f>'Overview'!V18</f>
             </strRef>
           </tx>
           <spPr>
@@ -594,12 +594,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overview'!$N$16</f>
+              <f>'Overview'!$W$16:$Z$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$N$18</f>
+              <f>'Overview'!$W$18:$Z$18</f>
             </numRef>
           </val>
         </ser>
@@ -608,7 +608,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Overview'!M19</f>
+              <f>'Overview'!V19</f>
             </strRef>
           </tx>
           <spPr>
@@ -618,12 +618,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overview'!$N$16</f>
+              <f>'Overview'!$W$16:$Z$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$N$19</f>
+              <f>'Overview'!$W$19:$Z$19</f>
             </numRef>
           </val>
         </ser>
@@ -632,7 +632,7 @@
           <order val="3"/>
           <tx>
             <strRef>
-              <f>'Overview'!M20</f>
+              <f>'Overview'!V20</f>
             </strRef>
           </tx>
           <spPr>
@@ -642,12 +642,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overview'!$N$16</f>
+              <f>'Overview'!$W$16:$Z$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$N$20</f>
+              <f>'Overview'!$W$20:$Z$20</f>
             </numRef>
           </val>
         </ser>
@@ -758,7 +758,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Overview'!Q24</f>
+              <f>'Overview'!AC24</f>
             </strRef>
           </tx>
           <spPr>
@@ -768,12 +768,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overview'!$R$23</f>
+              <f>'Overview'!$AD$23:$AG$23</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$R$24</f>
+              <f>'Overview'!$AD$24:$AG$24</f>
             </numRef>
           </val>
         </ser>
@@ -782,7 +782,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Overview'!Q25</f>
+              <f>'Overview'!AC25</f>
             </strRef>
           </tx>
           <spPr>
@@ -792,12 +792,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overview'!$R$23</f>
+              <f>'Overview'!$AD$23:$AG$23</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$R$25</f>
+              <f>'Overview'!$AD$25:$AG$25</f>
             </numRef>
           </val>
         </ser>
@@ -806,7 +806,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Overview'!Q26</f>
+              <f>'Overview'!AC26</f>
             </strRef>
           </tx>
           <spPr>
@@ -816,12 +816,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overview'!$R$23</f>
+              <f>'Overview'!$AD$23:$AG$23</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$R$26</f>
+              <f>'Overview'!$AD$26:$AG$26</f>
             </numRef>
           </val>
         </ser>
@@ -830,7 +830,7 @@
           <order val="3"/>
           <tx>
             <strRef>
-              <f>'Overview'!Q27</f>
+              <f>'Overview'!AC27</f>
             </strRef>
           </tx>
           <spPr>
@@ -840,12 +840,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overview'!$R$23</f>
+              <f>'Overview'!$AD$23:$AG$23</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$R$27</f>
+              <f>'Overview'!$AD$27:$AG$27</f>
             </numRef>
           </val>
         </ser>
@@ -955,7 +955,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Overview'!U6</f>
+              <f>'Overview'!AJ6</f>
             </strRef>
           </tx>
           <spPr>
@@ -973,12 +973,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$V$5</f>
+              <f>'Overview'!$AK$5:$AN$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$V$6</f>
+              <f>'Overview'!$AK$6:$AN$6</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -988,7 +988,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Overview'!U7</f>
+              <f>'Overview'!AJ7</f>
             </strRef>
           </tx>
           <spPr>
@@ -1006,12 +1006,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$V$5</f>
+              <f>'Overview'!$AK$5:$AN$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$V$7</f>
+              <f>'Overview'!$AK$7:$AN$7</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1021,7 +1021,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Overview'!U8</f>
+              <f>'Overview'!AJ8</f>
             </strRef>
           </tx>
           <spPr>
@@ -1039,12 +1039,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$V$5</f>
+              <f>'Overview'!$AK$5:$AN$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$V$8</f>
+              <f>'Overview'!$AK$8:$AN$8</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1054,7 +1054,7 @@
           <order val="3"/>
           <tx>
             <strRef>
-              <f>'Overview'!U9</f>
+              <f>'Overview'!AJ9</f>
             </strRef>
           </tx>
           <spPr>
@@ -1072,12 +1072,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$V$5</f>
+              <f>'Overview'!$AK$5:$AN$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$V$9</f>
+              <f>'Overview'!$AK$9:$AN$9</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1087,7 +1087,7 @@
           <order val="4"/>
           <tx>
             <strRef>
-              <f>'Overview'!U10</f>
+              <f>'Overview'!AJ10</f>
             </strRef>
           </tx>
           <spPr>
@@ -1105,12 +1105,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$V$5</f>
+              <f>'Overview'!$AK$5:$AN$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$V$10</f>
+              <f>'Overview'!$AK$10:$AN$10</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1120,7 +1120,7 @@
           <order val="5"/>
           <tx>
             <strRef>
-              <f>'Overview'!U11</f>
+              <f>'Overview'!AJ11</f>
             </strRef>
           </tx>
           <spPr>
@@ -1138,12 +1138,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$V$5</f>
+              <f>'Overview'!$AK$5:$AN$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$V$11</f>
+              <f>'Overview'!$AK$11:$AN$11</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1618,14 +1618,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V38"/>
+  <dimension ref="A1:AN38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col hidden="1" width="13" customWidth="1" min="5" max="5"/>
-    <col hidden="1" width="13" customWidth="1" min="6" max="6"/>
-    <col hidden="1" width="13" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col hidden="1" width="13" customWidth="1" min="8" max="8"/>
     <col hidden="1" width="13" customWidth="1" min="9" max="9"/>
     <col hidden="1" width="13" customWidth="1" min="10" max="10"/>
@@ -1641,6 +1641,24 @@
     <col hidden="1" width="13" customWidth="1" min="20" max="20"/>
     <col hidden="1" width="13" customWidth="1" min="21" max="21"/>
     <col hidden="1" width="13" customWidth="1" min="22" max="22"/>
+    <col hidden="1" width="13" customWidth="1" min="23" max="23"/>
+    <col hidden="1" width="13" customWidth="1" min="24" max="24"/>
+    <col hidden="1" width="13" customWidth="1" min="25" max="25"/>
+    <col hidden="1" width="13" customWidth="1" min="26" max="26"/>
+    <col hidden="1" width="13" customWidth="1" min="27" max="27"/>
+    <col hidden="1" width="13" customWidth="1" min="28" max="28"/>
+    <col hidden="1" width="13" customWidth="1" min="29" max="29"/>
+    <col hidden="1" width="13" customWidth="1" min="30" max="30"/>
+    <col hidden="1" width="13" customWidth="1" min="31" max="31"/>
+    <col hidden="1" width="13" customWidth="1" min="32" max="32"/>
+    <col hidden="1" width="13" customWidth="1" min="33" max="33"/>
+    <col hidden="1" width="13" customWidth="1" min="34" max="34"/>
+    <col hidden="1" width="13" customWidth="1" min="35" max="35"/>
+    <col hidden="1" width="13" customWidth="1" min="36" max="36"/>
+    <col hidden="1" width="13" customWidth="1" min="37" max="37"/>
+    <col hidden="1" width="13" customWidth="1" min="38" max="38"/>
+    <col hidden="1" width="13" customWidth="1" min="39" max="39"/>
+    <col hidden="1" width="13" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1675,12 +1693,57 @@
           <t>FY2024</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>FY2024</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
         <is>
           <t>FY2024</t>
         </is>
@@ -1695,20 +1758,38 @@
       <c r="B6" s="5" t="n">
         <v>17427943</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="C6" s="5" t="n">
+        <v>1352794</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>14552</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>106367</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>Total assets</t>
         </is>
       </c>
-      <c r="F6" t="n">
+      <c r="I6" t="n">
+        <v>106367</v>
+      </c>
+      <c r="J6" t="n">
+        <v>14552</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1352794</v>
+      </c>
+      <c r="L6" t="n">
         <v>17427943</v>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="AJ6" t="inlineStr">
         <is>
           <t>CET1 Ratio</t>
         </is>
       </c>
-      <c r="V6" t="n">
+      <c r="AN6" t="n">
         <v>418.5</v>
       </c>
     </row>
@@ -1721,20 +1802,38 @@
       <c r="B7" s="5" t="n">
         <v>1102894</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="C7" s="5" t="n">
+        <v>260524</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>50338</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>59537</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>Trade and other payables</t>
         </is>
       </c>
-      <c r="F7" t="n">
+      <c r="I7" t="n">
+        <v>59537</v>
+      </c>
+      <c r="J7" t="n">
+        <v>50338</v>
+      </c>
+      <c r="K7" t="n">
+        <v>260524</v>
+      </c>
+      <c r="L7" t="n">
         <v>1102894</v>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="AJ7" t="inlineStr">
         <is>
           <t>Tier 1 Ratio</t>
         </is>
       </c>
-      <c r="V7" t="n">
+      <c r="AN7" t="n">
         <v>418.5</v>
       </c>
     </row>
@@ -1747,30 +1846,48 @@
       <c r="B8" s="5" t="n">
         <v>15359865</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="C8" s="5" t="n">
+        <v>962179</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>-35786</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>46830</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>Total equity</t>
         </is>
       </c>
-      <c r="F8" t="n">
+      <c r="I8" t="n">
+        <v>46830</v>
+      </c>
+      <c r="J8" t="n">
+        <v>-35786</v>
+      </c>
+      <c r="K8" t="n">
+        <v>962179</v>
+      </c>
+      <c r="L8" t="n">
         <v>15359865</v>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="AJ8" t="inlineStr">
         <is>
           <t>Total Capital Ratio</t>
         </is>
       </c>
-      <c r="V8" t="n">
+      <c r="AN8" t="n">
         <v>418.5</v>
       </c>
     </row>
     <row r="9">
-      <c r="U9" t="inlineStr">
+      <c r="AJ9" t="inlineStr">
         <is>
           <t>Leverage Ratio</t>
         </is>
       </c>
-      <c r="V9" t="n">
+      <c r="AN9" t="n">
         <v>87.40000000000001</v>
       </c>
     </row>
@@ -1780,12 +1897,12 @@
           <t>Profit &amp; Loss Summary (£)</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="AJ10" t="inlineStr">
         <is>
           <t>LCR</t>
         </is>
       </c>
-      <c r="V10" t="n">
+      <c r="AN10" t="n">
         <v>999999</v>
       </c>
     </row>
@@ -1800,17 +1917,47 @@
           <t>FY2024</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
         <is>
           <t>FY2024</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="AJ11" t="inlineStr">
         <is>
           <t>NSFR</t>
         </is>
       </c>
-      <c r="V11" t="n">
+      <c r="AN11" t="n">
         <v>492.2</v>
       </c>
     </row>
@@ -1823,12 +1970,25 @@
       <c r="B12" s="5" t="n">
         <v>-6256733</v>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="C12" s="5" t="n">
+        <v>-1767933</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>-406751</v>
+      </c>
+      <c r="E12" s="5" t="n"/>
+      <c r="O12" t="inlineStr">
         <is>
           <t>Total operating expenses</t>
         </is>
       </c>
-      <c r="J12" t="n">
+      <c r="Q12" t="n">
+        <v>-406751</v>
+      </c>
+      <c r="R12" t="n">
+        <v>-1767933</v>
+      </c>
+      <c r="S12" t="n">
         <v>-6256733</v>
       </c>
     </row>
@@ -1841,12 +2001,25 @@
       <c r="B13" s="5" t="n">
         <v>-6193551</v>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="C13" s="5" t="n">
+        <v>-1769188</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>-406520</v>
+      </c>
+      <c r="E13" s="5" t="n"/>
+      <c r="O13" t="inlineStr">
         <is>
           <t>Loss for the year</t>
         </is>
       </c>
-      <c r="J13" t="n">
+      <c r="Q13" t="n">
+        <v>-406520</v>
+      </c>
+      <c r="R13" t="n">
+        <v>-1769188</v>
+      </c>
+      <c r="S13" t="n">
         <v>-6193551</v>
       </c>
     </row>
@@ -1868,7 +2041,37 @@
           <t>FY2024</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
         <is>
           <t>FY2024</t>
         </is>
@@ -1883,12 +2086,30 @@
       <c r="B17" s="5" t="n">
         <v>962179</v>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="C17" s="5" t="n">
+        <v>-35786</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>46830</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V17" t="inlineStr">
         <is>
           <t>Opening equity</t>
         </is>
       </c>
-      <c r="N17" t="n">
+      <c r="W17" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" t="n">
+        <v>46830</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>-35786</v>
+      </c>
+      <c r="Z17" t="n">
         <v>962179</v>
       </c>
     </row>
@@ -1901,12 +2122,30 @@
       <c r="B18" s="5" t="n">
         <v>-6126169</v>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="C18" s="5" t="n">
+        <v>-1769188</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>-406520</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>-219920</v>
+      </c>
+      <c r="V18" t="inlineStr">
         <is>
           <t>Total comprehensive income</t>
         </is>
       </c>
-      <c r="N18" t="n">
+      <c r="W18" t="n">
+        <v>-219920</v>
+      </c>
+      <c r="X18" t="n">
+        <v>-406520</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>-1769188</v>
+      </c>
+      <c r="Z18" t="n">
         <v>-6126169</v>
       </c>
     </row>
@@ -1919,12 +2158,30 @@
       <c r="B19" s="5" t="n">
         <v>20523855</v>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="C19" s="5" t="n">
+        <v>2767153</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>323904</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>266750</v>
+      </c>
+      <c r="V19" t="inlineStr">
         <is>
           <t>Other movements, net</t>
         </is>
       </c>
-      <c r="N19" t="n">
+      <c r="W19" t="n">
+        <v>266750</v>
+      </c>
+      <c r="X19" t="n">
+        <v>323904</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>2767153</v>
+      </c>
+      <c r="Z19" t="n">
         <v>20523855</v>
       </c>
     </row>
@@ -1937,12 +2194,30 @@
       <c r="B20" s="5" t="n">
         <v>15359865</v>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="C20" s="5" t="n">
+        <v>962179</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>-35786</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>46830</v>
+      </c>
+      <c r="V20" t="inlineStr">
         <is>
           <t>Closing equity</t>
         </is>
       </c>
-      <c r="N20" t="n">
+      <c r="W20" t="n">
+        <v>46830</v>
+      </c>
+      <c r="X20" t="n">
+        <v>-35786</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>962179</v>
+      </c>
+      <c r="Z20" t="n">
         <v>15359865</v>
       </c>
     </row>
@@ -1964,7 +2239,37 @@
           <t>FY2024</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="AG23" t="inlineStr">
         <is>
           <t>FY2024</t>
         </is>
@@ -1979,12 +2284,25 @@
       <c r="B24" s="5" t="n">
         <v>-5854403</v>
       </c>
-      <c r="Q24" t="inlineStr">
+      <c r="C24" s="5" t="n">
+        <v>-1747582</v>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>-402889</v>
+      </c>
+      <c r="E24" s="5" t="n"/>
+      <c r="AC24" t="inlineStr">
         <is>
           <t>Net cash outflow from operating activities</t>
         </is>
       </c>
-      <c r="R24" t="n">
+      <c r="AE24" t="n">
+        <v>-402889</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>-1747582</v>
+      </c>
+      <c r="AG24" t="n">
         <v>-5854403</v>
       </c>
     </row>
@@ -1997,12 +2315,25 @@
       <c r="B25" s="5" t="n">
         <v>-12345649</v>
       </c>
-      <c r="Q25" t="inlineStr">
+      <c r="C25" s="5" t="n">
+        <v>-31717</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="5" t="n"/>
+      <c r="AC25" t="inlineStr">
         <is>
           <t>Net cash used in investing activities</t>
         </is>
       </c>
-      <c r="R25" t="n">
+      <c r="AE25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>-31717</v>
+      </c>
+      <c r="AG25" t="n">
         <v>-12345649</v>
       </c>
     </row>
@@ -2015,12 +2346,25 @@
       <c r="B26" s="5" t="n">
         <v>20384295</v>
       </c>
-      <c r="Q26" t="inlineStr">
+      <c r="C26" s="5" t="n">
+        <v>2743644</v>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>323904</v>
+      </c>
+      <c r="E26" s="5" t="n"/>
+      <c r="AC26" t="inlineStr">
         <is>
           <t>Net cash generated from financing activities</t>
         </is>
       </c>
-      <c r="R26" t="n">
+      <c r="AE26" t="n">
+        <v>323904</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>2743644</v>
+      </c>
+      <c r="AG26" t="n">
         <v>20384295</v>
       </c>
     </row>
@@ -2033,12 +2377,30 @@
       <c r="B27" s="5" t="n">
         <v>3155921</v>
       </c>
-      <c r="Q27" t="inlineStr">
+      <c r="C27" s="5" t="n">
+        <v>971678</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>7333</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>86318</v>
+      </c>
+      <c r="AC27" t="inlineStr">
         <is>
           <t>Cash and cash equivalents at end of year</t>
         </is>
       </c>
-      <c r="R27" t="n">
+      <c r="AD27" t="n">
+        <v>86318</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>7333</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>971678</v>
+      </c>
+      <c r="AG27" t="n">
         <v>3155921</v>
       </c>
     </row>
@@ -2060,6 +2422,21 @@
           <t>FY2024</t>
         </is>
       </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -2072,6 +2449,21 @@
           <t>418.5%</t>
         </is>
       </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -2084,6 +2476,21 @@
           <t>418.5%</t>
         </is>
       </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -2096,6 +2503,21 @@
           <t>418.5%</t>
         </is>
       </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
@@ -2108,6 +2530,21 @@
           <t>87.4%</t>
         </is>
       </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
@@ -2120,6 +2557,21 @@
           <t>999999%</t>
         </is>
       </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -2132,17 +2584,32 @@
           <t>492.2%</t>
         </is>
       </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="45" customHeight="1">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>Note: SHORT PERIOD: This workbook intentionally covers FY2024 only. Afin's first Pillar 3 report states that it was authorised as a bank with restrictions in October 2024 and does not provide prior-period comparatives. The Pillar 3 metrics are standalone Afin Bank Limited disclosures; the cash-flow statement is from the audited annual accounts. See each detail sheet for the source citation. Asset Quality and RWA Breakdown are marked not publicly disclosed: Afin has no lending product on its balance sheet yet and, as a small non-complex institution, its Pillar 3 report has no exposure-class RWA table.</t>
+          <t>Note: EXTENDED HISTORY: this workbook now covers FY2021-FY2024 (four years), extended back from an original FY2024-only Pillar-3-only build. Afin Bank Limited was named All Africa Capital Limited and was not yet a PRA-authorised bank until October 2024, so FY2021-FY2023's Balance Sheet/P&amp;L/Equity/Cash Flow figures are that same continuous legal entity's own pre-bank Companies House statutory accounts, while all 11 Pillar 3 metric sheets plus Asset Quality and RWA Breakdown are genuinely 'Not applicable' for those three years (no disclosure obligation existed) - only FY2024 carries real Pillar 3 figures. FY2020 is self-skipped in full: the company was incorporated 18 December 2020 and its first statutory accounts cover the period from incorporation to 31 December 2021 - no discrete FY2020 period was ever filed, because none exists for this entity (confirmed by reading the complete Companies House filing history, not assumed from the entity-creation-date signal alone). FY2021's Profit &amp; Loss and Cash Flow Statement are themselves NOT DISCLOSED (small-companies filing exemptions - no P&amp;L account or cash flow statement was ever filed for that period); only its Balance Sheet and the equity roll-forward derived from it are available. Genuine structural findings, all documented on their own sheets: FY2023 is the first year with intangible assets, a lease/right-of-use asset, and an audit (FY2021-FY2022 were unaudited small-company filings); the FY2023 report's own 2022 comparative column is itself unaudited per its auditor's report. Every closing cash and equity balance ties exactly into the next year's own opening balance across all four years, including into the pre-existing FY2024 figures unchanged from the original build.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A38:E38"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2155,11 +2622,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2187,6 +2657,21 @@
           <t>FY2024</t>
         </is>
       </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2199,20 +2684,36 @@
           <t>418.5%</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="145" customHeight="1">
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="180" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
 FY2024: UK KM1 Key Metrics, printed pp. 4-5, and UK OV1, printed p. 5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
 Afin Bank annual reports and disclosures page - https://afinbank.com/about/annual-reports-and-disclosures/
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was incorporated 18 December 2020 as All Africa Capital Limited, traded under that name through FY2021-FY2023, and changed its name to Afin Bank Limited after receiving banking authorisation with restrictions in October 2024. FY2021-FY2023 figures below are therefore All Africa Capital Limited's own pre-bank statutory accounts for the same continuous legal entity, sourced from Companies House (not from afinbank.com, which only hosts the FY2024 bank-era documents).
+NOT APPLICABLE for FY2021-FY2023: All Africa Capital Limited (this entity's name before October 2024) was not a PRA-authorised bank during FY2021-FY2023 and had no Pillar 3 disclosure obligation - its own filed accounts for those years contain no capital/liquidity/leverage/RWA figures of any kind. This is a genuine 'not applicable' (no obligation existed), distinct from 'not publicly disclosed' (an obligated but unpublished figure), which is how FY2024's own non-disclosures are marked.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A6:E6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2224,11 +2725,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2256,6 +2760,21 @@
           <t>FY2024</t>
         </is>
       </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2266,20 +2785,36 @@
       <c r="B4" s="6" t="n">
         <v>12922</v>
       </c>
-    </row>
-    <row r="6" ht="145" customHeight="1">
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="180" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
 FY2024: UK KM1 Key Metrics, printed pp. 4-5, and UK OV1, printed p. 5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
 Afin Bank annual reports and disclosures page - https://afinbank.com/about/annual-reports-and-disclosures/
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was incorporated 18 December 2020 as All Africa Capital Limited, traded under that name through FY2021-FY2023, and changed its name to Afin Bank Limited after receiving banking authorisation with restrictions in October 2024. FY2021-FY2023 figures below are therefore All Africa Capital Limited's own pre-bank statutory accounts for the same continuous legal entity, sourced from Companies House (not from afinbank.com, which only hosts the FY2024 bank-era documents).
+NOT APPLICABLE for FY2021-FY2023: All Africa Capital Limited (this entity's name before October 2024) was not a PRA-authorised bank during FY2021-FY2023 and had no Pillar 3 disclosure obligation - its own filed accounts for those years contain no capital/liquidity/leverage/RWA figures of any kind. This is a genuine 'not applicable' (no obligation existed), distinct from 'not publicly disclosed' (an obligated but unpublished figure), which is how FY2024's own non-disclosures are marked.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A6:E6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2291,11 +2826,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2323,6 +2861,21 @@
           <t>FY2024</t>
         </is>
       </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2335,20 +2888,36 @@
           <t>418.5%</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="145" customHeight="1">
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="180" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
 FY2024: UK KM1 Key Metrics, printed pp. 4-5, and UK OV1, printed p. 5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
 Afin Bank annual reports and disclosures page - https://afinbank.com/about/annual-reports-and-disclosures/
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was incorporated 18 December 2020 as All Africa Capital Limited, traded under that name through FY2021-FY2023, and changed its name to Afin Bank Limited after receiving banking authorisation with restrictions in October 2024. FY2021-FY2023 figures below are therefore All Africa Capital Limited's own pre-bank statutory accounts for the same continuous legal entity, sourced from Companies House (not from afinbank.com, which only hosts the FY2024 bank-era documents).
+NOT APPLICABLE for FY2021-FY2023: All Africa Capital Limited (this entity's name before October 2024) was not a PRA-authorised bank during FY2021-FY2023 and had no Pillar 3 disclosure obligation - its own filed accounts for those years contain no capital/liquidity/leverage/RWA figures of any kind. This is a genuine 'not applicable' (no obligation existed), distinct from 'not publicly disclosed' (an obligated but unpublished figure), which is how FY2024's own non-disclosures are marked.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A6:E6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2360,11 +2929,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2392,6 +2964,21 @@
           <t>FY2024</t>
         </is>
       </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2402,20 +2989,36 @@
       <c r="B4" s="6" t="n">
         <v>3087</v>
       </c>
-    </row>
-    <row r="6" ht="145" customHeight="1">
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="180" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
 FY2024: UK KM1 Key Metrics, printed pp. 4-5, and UK OV1, printed p. 5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
 Afin Bank annual reports and disclosures page - https://afinbank.com/about/annual-reports-and-disclosures/
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was incorporated 18 December 2020 as All Africa Capital Limited, traded under that name through FY2021-FY2023, and changed its name to Afin Bank Limited after receiving banking authorisation with restrictions in October 2024. FY2021-FY2023 figures below are therefore All Africa Capital Limited's own pre-bank statutory accounts for the same continuous legal entity, sourced from Companies House (not from afinbank.com, which only hosts the FY2024 bank-era documents).
+NOT APPLICABLE for FY2021-FY2023: All Africa Capital Limited (this entity's name before October 2024) was not a PRA-authorised bank during FY2021-FY2023 and had no Pillar 3 disclosure obligation - its own filed accounts for those years contain no capital/liquidity/leverage/RWA figures of any kind. This is a genuine 'not applicable' (no obligation existed), distinct from 'not publicly disclosed' (an obligated but unpublished figure), which is how FY2024's own non-disclosures are marked.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A6:E6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2427,11 +3030,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2459,32 +3065,63 @@
           <t>FY2024 (£'000)</t>
         </is>
       </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>FY2023 (£'000)</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>FY2022 (£'000)</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FY2021 (£'000)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
+          <t>Not publicly disclosed / Not applicable</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
           <t>Not publicly disclosed</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Not publicly disclosed</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="150" customHeight="1">
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="180" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
 UK KM1 Key Metrics, printed pp. 4-5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.
-NOT DISCLOSED: as a small non-complex institution under CRR Article 433b, Afin Bank's 2024 Pillar 3 disclosure contains only the single aggregate Total RWA figure in UK KM1 (see the Total RWAs sheet) - no UK OV1 exposure-class breakdown is published.</t>
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was incorporated 18 December 2020 as All Africa Capital Limited, traded under that name through FY2021-FY2023, and changed its name to Afin Bank Limited after receiving banking authorisation with restrictions in October 2024. FY2021-FY2023 figures below are therefore All Africa Capital Limited's own pre-bank statutory accounts for the same continuous legal entity, sourced from Companies House (not from afinbank.com, which only hosts the FY2024 bank-era documents).
+NOT DISCLOSED (FY2024): as a small non-complex institution under CRR Article 433b, Afin Bank's 2024 Pillar 3 disclosure contains only the single aggregate Total RWA figure in UK KM1 (see the Total RWAs sheet) - no UK OV1 exposure-class breakdown is published.
+NOT APPLICABLE for FY2021-FY2023: All Africa Capital Limited (this entity's name before October 2024) was not a PRA-authorised bank during FY2021-FY2023 and had no Pillar 3 disclosure obligation - its own filed accounts for those years contain no capital/liquidity/leverage/RWA figures of any kind. This is a genuine 'not applicable' (no obligation existed), distinct from 'not publicly disclosed' (an obligated but unpublished figure), which is how FY2024's own non-disclosures are marked.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A6:E6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2496,11 +3133,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2528,6 +3168,21 @@
           <t>FY2024</t>
         </is>
       </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2538,6 +3193,21 @@
       <c r="B4" s="6" t="n">
         <v>14782</v>
       </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2550,20 +3220,36 @@
           <t>87.4%</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="145" customHeight="1">
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="180" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
 FY2024: UK KM1 Key Metrics, printed pp. 4-5, and UK OV1, printed p. 5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
 Afin Bank annual reports and disclosures page - https://afinbank.com/about/annual-reports-and-disclosures/
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was incorporated 18 December 2020 as All Africa Capital Limited, traded under that name through FY2021-FY2023, and changed its name to Afin Bank Limited after receiving banking authorisation with restrictions in October 2024. FY2021-FY2023 figures below are therefore All Africa Capital Limited's own pre-bank statutory accounts for the same continuous legal entity, sourced from Companies House (not from afinbank.com, which only hosts the FY2024 bank-era documents).
+NOT APPLICABLE for FY2021-FY2023: All Africa Capital Limited (this entity's name before October 2024) was not a PRA-authorised bank during FY2021-FY2023 and had no Pillar 3 disclosure obligation - its own filed accounts for those years contain no capital/liquidity/leverage/RWA figures of any kind. This is a genuine 'not applicable' (no obligation existed), distinct from 'not publicly disclosed' (an obligated but unpublished figure), which is how FY2024's own non-disclosures are marked.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A7:E7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2575,11 +3261,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2607,6 +3296,21 @@
           <t>FY2024</t>
         </is>
       </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2617,6 +3321,21 @@
       <c r="B4" s="6" t="n">
         <v>8909</v>
       </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2627,6 +3346,21 @@
       <c r="B5" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2637,6 +3371,21 @@
       <c r="B6" s="6" t="n">
         <v>3971</v>
       </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2647,6 +3396,21 @@
       <c r="B7" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -2659,28 +3423,44 @@
           <t>999999%</t>
         </is>
       </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="60" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Note: Afin states that it had no qualifying cash outflows at 31 December 2024; the source therefore reports the LCR as 999999%. This is reproduced as reported and is not interpreted as a conventional finite ratio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="145" customHeight="1">
+          <t>Note: Afin states that it had no qualifying cash outflows at 31 December 2024; the source therefore reports the LCR as 999999%. This is reproduced as reported and is not interpreted as a conventional finite ratio. FY2021-FY2023 predate Afin's banking authorisation - no LCR obligation existed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="180" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
 FY2024: UK KM1 Key Metrics, printed pp. 4-5, and UK OV1, printed p. 5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
 Afin Bank annual reports and disclosures page - https://afinbank.com/about/annual-reports-and-disclosures/
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was incorporated 18 December 2020 as All Africa Capital Limited, traded under that name through FY2021-FY2023, and changed its name to Afin Bank Limited after receiving banking authorisation with restrictions in October 2024. FY2021-FY2023 figures below are therefore All Africa Capital Limited's own pre-bank statutory accounts for the same continuous legal entity, sourced from Companies House (not from afinbank.com, which only hosts the FY2024 bank-era documents).
+NOT APPLICABLE for FY2021-FY2023: All Africa Capital Limited (this entity's name before October 2024) was not a PRA-authorised bank during FY2021-FY2023 and had no Pillar 3 disclosure obligation - its own filed accounts for those years contain no capital/liquidity/leverage/RWA figures of any kind. This is a genuine 'not applicable' (no obligation existed), distinct from 'not publicly disclosed' (an obligated but unpublished figure), which is how FY2024's own non-disclosures are marked.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A9:E9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2692,11 +3472,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2724,6 +3507,21 @@
           <t>FY2024</t>
         </is>
       </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -2734,6 +3532,21 @@
       <c r="B4" s="6" t="n">
         <v>21486</v>
       </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2744,6 +3557,21 @@
       <c r="B5" s="6" t="n">
         <v>4365</v>
       </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2756,20 +3584,36 @@
           <t>492.2%</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="145" customHeight="1">
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="180" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
 FY2024: UK KM1 Key Metrics, printed pp. 4-5, and UK OV1, printed p. 5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
 Afin Bank annual reports and disclosures page - https://afinbank.com/about/annual-reports-and-disclosures/
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was incorporated 18 December 2020 as All Africa Capital Limited, traded under that name through FY2021-FY2023, and changed its name to Afin Bank Limited after receiving banking authorisation with restrictions in October 2024. FY2021-FY2023 figures below are therefore All Africa Capital Limited's own pre-bank statutory accounts for the same continuous legal entity, sourced from Companies House (not from afinbank.com, which only hosts the FY2024 bank-era documents).
+NOT APPLICABLE for FY2021-FY2023: All Africa Capital Limited (this entity's name before October 2024) was not a PRA-authorised bank during FY2021-FY2023 and had no Pillar 3 disclosure obligation - its own filed accounts for those years contain no capital/liquidity/leverage/RWA figures of any kind. This is a genuine 'not applicable' (no obligation existed), distinct from 'not publicly disclosed' (an obligated but unpublished figure), which is how FY2024's own non-disclosures are marked.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A8:E8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2781,11 +3625,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2809,40 +3656,71 @@
           <t>FY2024</t>
         </is>
       </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>MREL Ratio</t>
+          <t>MREL ratio</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Not publicly disclosed</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Note: No numeric MREL ratio is disclosed in the 2024 Pillar 3 report or the audited annual accounts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="150" customHeight="1">
+          <t>Note: No numeric MREL ratio is disclosed in the 2024 Pillar 3 report or the audited annual accounts for FY2024. FY2021-FY2023 predate Afin's banking authorisation (October 2024), so no MREL obligation existed for those years.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="180" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
 FY2024: UK KM1 Key Metrics, printed pp. 4-5, and UK OV1, printed p. 5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
 Afin Bank annual reports and disclosures page - https://afinbank.com/about/annual-reports-and-disclosures/
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was incorporated 18 December 2020 as All Africa Capital Limited, traded under that name through FY2021-FY2023, and changed its name to Afin Bank Limited after receiving banking authorisation with restrictions in October 2024. FY2021-FY2023 figures below are therefore All Africa Capital Limited's own pre-bank statutory accounts for the same continuous legal entity, sourced from Companies House (not from afinbank.com, which only hosts the FY2024 bank-era documents).
+NOT APPLICABLE for FY2021-FY2023: All Africa Capital Limited (this entity's name before October 2024) was not a PRA-authorised bank during FY2021-FY2023 and had no Pillar 3 disclosure obligation - its own filed accounts for those years contain no capital/liquidity/leverage/RWA figures of any kind. This is a genuine 'not applicable' (no obligation existed), distinct from 'not publicly disclosed' (an obligated but unpublished figure), which is how FY2024's own non-disclosures are marked.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A7:E7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2854,11 +3732,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2871,7 +3752,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Afin Bank Limited audited statement of financial position; amounts in £.</t>
+          <t>Afin Bank Limited (All Africa Capital Limited pre-October 2024) audited/unaudited statement of financial position; amounts in £. FY2021 covers the first accounting period, 18 Dec 2020-31 Dec 2021 (FY2020 does not exist as a discrete period - see source note).</t>
         </is>
       </c>
     </row>
@@ -2886,6 +3767,21 @@
           <t>FY2024 (£)</t>
         </is>
       </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>FY2023 (£)</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>FY2022 (£)</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FY2021 (£)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -2894,6 +3790,9 @@
         </is>
       </c>
       <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2904,6 +3803,15 @@
       <c r="B5" s="6" t="n">
         <v>3155921</v>
       </c>
+      <c r="C5" s="6" t="n">
+        <v>971678</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>7333</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>86318</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2914,6 +3822,9 @@
       <c r="B6" s="6" t="n">
         <v>9767797</v>
       </c>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2924,6 +3835,15 @@
       <c r="B7" s="6" t="n">
         <v>450628</v>
       </c>
+      <c r="C7" s="6" t="n">
+        <v>166804</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>6859</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>19562</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -2934,6 +3854,13 @@
       <c r="B8" s="6" t="n">
         <v>372022</v>
       </c>
+      <c r="C8" s="6" t="n">
+        <v>50123</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -2944,6 +3871,15 @@
       <c r="B9" s="6" t="n">
         <v>57172</v>
       </c>
+      <c r="C9" s="6" t="n">
+        <v>152189</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>360</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>487</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -2954,6 +3890,9 @@
       <c r="B10" s="6" t="n">
         <v>967204</v>
       </c>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -2964,6 +3903,11 @@
       <c r="B11" s="6" t="n">
         <v>2657199</v>
       </c>
+      <c r="C11" s="6" t="n">
+        <v>12000</v>
+      </c>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -2974,6 +3918,15 @@
       <c r="B12" s="5" t="n">
         <v>17427943</v>
       </c>
+      <c r="C12" s="5" t="n">
+        <v>1352794</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>14552</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>106367</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -2982,6 +3935,9 @@
         </is>
       </c>
       <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -2992,6 +3948,15 @@
       <c r="B14" s="6" t="n">
         <v>1102894</v>
       </c>
+      <c r="C14" s="6" t="n">
+        <v>260524</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>50338</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>59537</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -3002,6 +3967,13 @@
       <c r="B15" s="6" t="n">
         <v>965184</v>
       </c>
+      <c r="C15" s="6" t="n">
+        <v>130091</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -3012,6 +3984,15 @@
       <c r="B16" s="5" t="n">
         <v>2068078</v>
       </c>
+      <c r="C16" s="5" t="n">
+        <v>390615</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>50338</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>59537</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -3022,6 +4003,15 @@
       <c r="B17" s="5" t="n">
         <v>15359865</v>
       </c>
+      <c r="C17" s="5" t="n">
+        <v>962179</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>-35786</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>46830</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -3030,6 +4020,9 @@
         </is>
       </c>
       <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -3040,6 +4033,15 @@
       <c r="B19" s="6" t="n">
         <v>23614036</v>
       </c>
+      <c r="C19" s="6" t="n">
+        <v>3357807</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>590654</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>266750</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -3050,6 +4052,9 @@
       <c r="B20" s="6" t="n">
         <v>67382</v>
       </c>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -3060,6 +4065,9 @@
       <c r="B21" s="6" t="n">
         <v>267626</v>
       </c>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -3070,6 +4078,15 @@
       <c r="B22" s="6" t="n">
         <v>-8589179</v>
       </c>
+      <c r="C22" s="6" t="n">
+        <v>-2395628</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>-626440</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>-219920</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -3080,20 +4097,32 @@
       <c r="B23" s="5" t="n">
         <v>15359865</v>
       </c>
-    </row>
-    <row r="25" ht="150" customHeight="1">
+      <c r="C23" s="5" t="n">
+        <v>962179</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>-35786</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>46830</v>
+      </c>
+    </row>
+    <row r="25" ht="210" customHeight="1">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>Sources - Afin Bank Limited audited annual report and financial statements for the year ended 31 December 2024:
-FY2024: Statement of financial position, printed p. 34 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-Ltd-Year-End-Accounts-FV24-FINAL-SIGNED.pdf
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.
-PRESENTATION NOTE: The source statement also shows FY2023 comparatives on its face, but this workbook is intentionally FY2024-only for consistency with the Cash Flow Statement and Pillar 3 sheets, whose primary source (the 2024 Pillar 3 report) explicitly states no prior-period comparatives are provided.</t>
+          <t>Sources - FY2024: Afin Bank Limited audited annual report and financial statements for the year ended 31 December 2024, statement of financial position, printed p. 34 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-Ltd-Year-End-Accounts-FV24-FINAL-SIGNED.pdf
+FY2023: All Africa Capital Limited audited annual report and financial statements for the year ended 31 December 2023, statement of financial position, p. 7 (2023 column; 2022 comparative column) - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history/MzQyNDA1MjMwOGFkaXF6a2N4/document?format=pdf&amp;download=0
+FY2022: All Africa Capital Limited unaudited financial statements for the year ended 31 December 2022, balance sheet, p. 1 (cross-checked against the FY2023 report's own 2022 comparative - ties exactly) - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history/MzM5MzI3MzYzNmFkaXF6a2N4/document?format=pdf&amp;download=0
+FY2021: All Africa Capital Limited unaudited financial statements for the period ended 31 December 2021 (first accounting period, from incorporation 18 December 2020), balance sheet, p. 1 - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history/MzM2MjY4Mzc2MGFkaXF6a2N4/document?format=pdf&amp;download=0
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was incorporated 18 December 2020 as All Africa Capital Limited, traded under that name through FY2021-FY2023, and changed its name to Afin Bank Limited after receiving banking authorisation with restrictions in October 2024. FY2021-FY2023 figures below are therefore All Africa Capital Limited's own pre-bank statutory accounts for the same continuous legal entity, sourced from Companies House (not from afinbank.com, which only hosts the FY2024 bank-era documents).
+STRUCTURAL NOTES: (1) 'Treasury assets', 'Right-of-use assets', 'Revaluation reserve' and 'Share based payment reserve' are all genuinely new line items that first appear on the FY2024 face statement (post-banking-authorisation) - left blank, not zero, for FY2021-FY2023, where the underlying asset/liability class simply did not exist on the company's books. (2) FY2023's face statement combines right-of-use assets into the single 'Property, plant and equipment' line (its own note 10 breaks out Computer equipment £22,098 + Right of use asset £130,091 = £152,189); FY2022/FY2021 predate IFRS 16 entirely (no leases). (3) FY2021's 'Debtors' £19,562 is a single undifferentiated line (no prepayments split existed yet) - reproduced under 'Receivables' with FY2021's own 'Prepayments' cell left blank rather than zero. (4) 'Receivables' for FY2023 combines the current £147,604 and non-current £19,200 other-receivables notes into one face-equivalent figure, consistent with how FY2024's own single 'Receivables' row is presented.
+FY2020 SELF-SKIPPED IN FULL: the company was incorporated 18 December 2020, so no financial year beginning 1 January 2020 exists for this entity, and no such period was ever filed at Companies House. Its first statutory accounts (filed 16 December 2022) cover the period from incorporation (18 December 2020) to 31 December 2021 - a single ~13.5-month first accounting period, not a discrete FY2020 followed by a discrete FY2021. This was confirmed by reading the full Companies House filing history for company 13090556 (all 4 pages, back to incorporation), not assumed from the entity-creation-date signal alone - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A25:E25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3105,11 +4134,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3122,7 +4154,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Afin Bank Limited audited statement of comprehensive income; amounts in £.</t>
+          <t>Afin Bank Limited (All Africa Capital Limited pre-October 2024) audited/unaudited statement of comprehensive income; amounts in £. FY2021 NOT DISCLOSED (small-companies exemption - see source note).</t>
         </is>
       </c>
     </row>
@@ -3137,176 +4169,363 @@
           <t>FY2024 (£)</t>
         </is>
       </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>FY2023 (£)</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>FY2022 (£)</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FY2021 (£)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Operating expenses</t>
+          <t>Operating income and expenses</t>
         </is>
       </c>
       <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Staff costs</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n">
-        <v>-3941455</v>
-      </c>
+          <t>Other operating income</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>231</v>
+      </c>
+      <c r="E5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Depreciation</t>
+          <t>Staff costs</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>-142504</v>
-      </c>
+        <v>-3941455</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>-1088800</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>-224067</v>
+      </c>
+      <c r="E6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Amortisation of intangibles</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
-        <v>-23179</v>
-      </c>
+          <t>Computer running costs</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n">
+        <v>-45103</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>-3026</v>
+      </c>
+      <c r="E7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Other operating costs</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>-2149595</v>
-      </c>
+          <t>Legal and professional fees</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n">
+        <v>-166504</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>-42042</v>
+      </c>
+      <c r="E8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Total operating expenses</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>-6256733</v>
-      </c>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Consultancy fees</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n">
+        <v>-276803</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>-123016</v>
+      </c>
+      <c r="E9" s="6" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Operating loss</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n">
-        <v>-6256733</v>
-      </c>
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Audit fees</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n">
+        <v>-8760</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Finance income</t>
+          <t>Depreciation</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>75152</v>
-      </c>
+        <v>-142504</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>-21488</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>-127</v>
+      </c>
+      <c r="E11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Finance costs</t>
+          <t>Amortisation of intangibles</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>-11970</v>
-      </c>
+        <v>-23179</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Loss before taxation</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="n">
-        <v>-6193551</v>
-      </c>
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Other operating costs</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>-2149595</v>
+      </c>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Income tax expense</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="n">
-        <v>0</v>
-      </c>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Total operating expenses</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>-6256733</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>-1767933</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>-406751</v>
+      </c>
+      <c r="E14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Loss for the year</t>
+          <t>Operating loss</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>-6193551</v>
-      </c>
+        <v>-6256733</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>-1767933</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>-406520</v>
+      </c>
+      <c r="E15" s="5" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Other comprehensive income</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="n"/>
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Finance income</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>75152</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Treasury asset revaluation</t>
+          <t>Finance costs</t>
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>67382</v>
-      </c>
+        <v>-11970</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>-1263</v>
+      </c>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
+          <t>Loss before taxation</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>-6193551</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>-1769188</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>-406520</v>
+      </c>
+      <c r="E18" s="5" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Income tax expense</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Loss for the year</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>-6193551</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>-1769188</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>-406520</v>
+      </c>
+      <c r="E20" s="5" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Other comprehensive income</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Treasury asset revaluation</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n">
+        <v>67382</v>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
           <t>Total other comprehensive income for the year</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n">
+      <c r="B23" s="5" t="n">
         <v>67382</v>
       </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="C23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="5" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Total comprehensive income for the year</t>
         </is>
       </c>
-      <c r="B19" s="5" t="n">
+      <c r="B24" s="5" t="n">
         <v>-6126169</v>
       </c>
-    </row>
-    <row r="21" ht="150" customHeight="1">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>Sources - Afin Bank Limited audited annual report and financial statements for the year ended 31 December 2024:
-FY2024: Statement of comprehensive income, printed p. 33 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-Ltd-Year-End-Accounts-FV24-FINAL-SIGNED.pdf
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.
-PRESENTATION NOTE: The source statement also shows FY2023 comparatives on its face, but this workbook is intentionally FY2024-only for consistency with the Cash Flow Statement and Pillar 3 sheets.</t>
+      <c r="C24" s="5" t="n">
+        <v>-1769188</v>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>-406520</v>
+      </c>
+      <c r="E24" s="5" t="n"/>
+    </row>
+    <row r="26" ht="210" customHeight="1">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>Sources - FY2024: Afin Bank Limited audited annual report and financial statements for the year ended 31 December 2024, statement of comprehensive income, printed p. 33 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-Ltd-Year-End-Accounts-FV24-FINAL-SIGNED.pdf
+FY2023: All Africa Capital Limited audited annual report and financial statements for the year ended 31 December 2023, statement of comprehensive income p. 6 and operating loss note 5 p. 14 (2023 column; 2022 comparative column, itself unaudited) - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history/MzQyNDA1MjMwOGFkaXF6a2N4/document?format=pdf&amp;download=0
+FY2022: as above (FY2023 report's own 2022 comparative and note 5 breakdown - the standalone FY2022 filing states the directors elected not to include a P&amp;L account within the filed financial statements) - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history/MzM5MzI3MzYzNmFkaXF6a2N4/document?format=pdf&amp;download=0
+FY2021: NOT DISCLOSED - the directors of All Africa Capital Limited elected not to include a copy of the profit and loss account within the filed financial statements for the period ended 31 December 2021 (a small-companies filing exemption); no P&amp;L breakdown exists in any source reviewed - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history/MzM2MjY4Mzc2MGFkaXF6a2N4/document?format=pdf&amp;download=0
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was incorporated 18 December 2020 as All Africa Capital Limited, traded under that name through FY2021-FY2023, and changed its name to Afin Bank Limited after receiving banking authorisation with restrictions in October 2024. FY2021-FY2023 figures below are therefore All Africa Capital Limited's own pre-bank statutory accounts for the same continuous legal entity, sourced from Companies House (not from afinbank.com, which only hosts the FY2024 bank-era documents).
+STRUCTURAL NOTE: FY2023/FY2022's own administrative-expenses note (note 5) splits costs as Staff costs / Computer running costs / Legal and professional fees / Consultancy fees / Audit fees / Depreciation / Other costs and separately discloses 'Other operating income' (£231 in FY2022, £nil in FY2023) - reproduced as its own set of rows rather than force-mapped onto FY2024's differently-labelled 'Other operating costs' bucket. Both years' figures were verified to foot exactly to the reported Administrative expenses total.
+FY2020 SELF-SKIPPED IN FULL: the company was incorporated 18 December 2020, so no financial year beginning 1 January 2020 exists for this entity, and no such period was ever filed at Companies House. Its first statutory accounts (filed 16 December 2022) cover the period from incorporation (18 December 2020) to 31 December 2021 - a single ~13.5-month first accounting period, not a discrete FY2020 followed by a discrete FY2021. This was confirmed by reading the full Companies House filing history for company 13090556 (all 4 pages, back to incorporation), not assumed from the entity-creation-date signal alone - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A26:E26"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3318,7 +4537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3339,7 +4558,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Afin Bank Limited audited statement of changes in equity, 1 January 2023 to 31 December 2024; amounts in £.</t>
+          <t>Afin Bank Limited (All Africa Capital Limited pre-October 2024) statement of changes in equity, 18 December 2020 (incorporation) to 31 December 2024; amounts in £.</t>
         </is>
       </c>
     </row>
@@ -3378,61 +4597,61 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Balance at 1 January 2023</t>
+          <t>Balance at 18 December 2020 (date of incorporation)</t>
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>590654</v>
+        <v>0</v>
       </c>
       <c r="C4" s="5" t="n"/>
       <c r="D4" s="5" t="n"/>
       <c r="E4" s="5" t="n">
-        <v>-626440</v>
+        <v>0</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>-35786</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Total comprehensive income for the year (2023)</t>
+          <t>Total comprehensive income for the period (18 Dec 2020 to 31 Dec 2021)</t>
         </is>
       </c>
       <c r="B5" s="6" t="n"/>
       <c r="C5" s="6" t="n"/>
       <c r="D5" s="6" t="n"/>
       <c r="E5" s="6" t="n">
-        <v>-1769188</v>
+        <v>-219920</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>-1769188</v>
+        <v>-219920</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Issue of share capital (2023)</t>
+          <t>Issue of share capital (2021)</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>2767153</v>
+        <v>266750</v>
       </c>
       <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n">
-        <v>2767153</v>
+        <v>266750</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Balance at 31 December 2023</t>
+          <t>Balance at 31 December 2021</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>3357807</v>
+        <v>266750</v>
       </c>
       <c r="C7" s="5" t="n">
         <v>0</v>
@@ -3441,129 +4660,234 @@
         <v>0</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>-2395628</v>
+        <v>-219920</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>962179</v>
+        <v>46830</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Loss for the year (2024)</t>
+          <t>Total comprehensive income for the year (2022)</t>
         </is>
       </c>
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
       <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="n">
-        <v>-6193551</v>
+        <v>-406520</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>-6193551</v>
+        <v>-406520</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Other comprehensive income - Treasury asset revaluation (2024)</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n">
-        <v>67382</v>
-      </c>
+          <t>Issue of share capital (2022)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>323904</v>
+      </c>
+      <c r="C9" s="6" t="n"/>
       <c r="D9" s="6" t="n"/>
       <c r="E9" s="6" t="n"/>
       <c r="F9" s="6" t="n">
-        <v>67382</v>
+        <v>323904</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Total comprehensive income for the year (2024)</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n">
-        <v>67382</v>
-      </c>
+          <t>Balance at 1 January 2023</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>590654</v>
+      </c>
+      <c r="C10" s="5" t="n"/>
       <c r="D10" s="5" t="n"/>
       <c r="E10" s="5" t="n">
-        <v>-6193551</v>
+        <v>-626440</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>-6126169</v>
+        <v>-35786</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Issue of share capital (2024)</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n">
-        <v>20256229</v>
-      </c>
+          <t>Total comprehensive income for the year (2023)</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n"/>
       <c r="C11" s="6" t="n"/>
       <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
+      <c r="E11" s="6" t="n">
+        <v>-1769188</v>
+      </c>
       <c r="F11" s="6" t="n">
-        <v>20256229</v>
+        <v>-1769188</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Share based payment (2024)</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="n"/>
+          <t>Issue of share capital (2023)</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>2767153</v>
+      </c>
       <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n">
-        <v>267626</v>
-      </c>
+      <c r="D12" s="6" t="n"/>
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="6" t="n">
-        <v>267626</v>
+        <v>2767153</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
+          <t>Balance at 31 December 2023</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>3357807</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>-2395628</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>962179</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Loss for the year (2024)</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n">
+        <v>-6193551</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>-6193551</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Other comprehensive income - Treasury asset revaluation (2024)</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n">
+        <v>67382</v>
+      </c>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n">
+        <v>67382</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Total comprehensive income for the year (2024)</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="5" t="n">
+        <v>67382</v>
+      </c>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5" t="n">
+        <v>-6193551</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>-6126169</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Issue of share capital (2024)</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>20256229</v>
+      </c>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n">
+        <v>20256229</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Share based payment (2024)</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n">
+        <v>267626</v>
+      </c>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n">
+        <v>267626</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
           <t>Balance at 31 December 2024</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n">
+      <c r="B19" s="5" t="n">
         <v>23614036</v>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C19" s="5" t="n">
         <v>67382</v>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D19" s="5" t="n">
         <v>267626</v>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E19" s="5" t="n">
         <v>-8589179</v>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="F19" s="5" t="n">
         <v>15359865</v>
       </c>
     </row>
-    <row r="15" ht="150" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>Sources - Afin Bank Limited audited annual report and financial statements for the year ended 31 December 2024:
-Statement of changes in equity, printed p. 35, covering 1 January 2023 to 31 December 2024 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-Ltd-Year-End-Accounts-FV24-FINAL-SIGNED.pdf
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.
-This is the one sheet in the workbook that includes FY2023 movements, since the equity roll-forward is chronological (not year-columned) and both years' movements are disclosed on the statement's face.</t>
+    <row r="21" ht="210" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Sources - FY2024: Afin Bank Limited audited annual report and financial statements for the year ended 31 December 2024, statement of changes in equity, p. 35, covering 1 January 2023 to 31 December 2024 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-Ltd-Year-End-Accounts-FV24-FINAL-SIGNED.pdf
+FY2021-FY2023: All Africa Capital Limited's own statement of changes in equity (FY2023 report, p. 8, covering 1 January 2022 to 31 December 2023) - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history/MzQyNDA1MjMwOGFkaXF6a2N4/document?format=pdf&amp;download=0 - plus the FY2021 first-period balance sheet (opening/closing bridge derived from its own reported balances) - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history/MzM2MjY4Mzc2MGFkaXF6a2N4/document?format=pdf&amp;download=0
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was incorporated 18 December 2020 as All Africa Capital Limited, traded under that name through FY2021-FY2023, and changed its name to Afin Bank Limited after receiving banking authorisation with restrictions in October 2024. FY2021-FY2023 figures below are therefore All Africa Capital Limited's own pre-bank statutory accounts for the same continuous legal entity, sourced from Companies House (not from afinbank.com, which only hosts the FY2024 bank-era documents).
+This sheet now runs chronologically from incorporation (18 December 2020) through 31 December 2024, the one sheet in the workbook not self-skipping FY2020: even though no discrete FY2020 accounts exist (see FY2020_SKIP_NOTE), the equity roll-forward correctly shows the company's true opening position at incorporation (£0) as its own row, with the first accounting period's entire movement (18 December 2020 to 31 December 2021) shown as a single aggregate line - the small-companies filing exemption from including a P&amp;L account means no finer split of that movement is available from any source.
+FY2020 SELF-SKIPPED IN FULL: the company was incorporated 18 December 2020, so no financial year beginning 1 January 2020 exists for this entity, and no such period was ever filed at Companies House. Its first statutory accounts (filed 16 December 2022) cover the period from incorporation (18 December 2020) to 31 December 2021 - a single ~13.5-month first accounting period, not a discrete FY2020 followed by a discrete FY2021. This was confirmed by reading the full Companies House filing history for company 13090556 (all 4 pages, back to incorporation), not assumed from the entity-creation-date signal alone - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A21:F21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3575,11 +4899,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3592,7 +4919,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Afin Bank Limited audited standalone statement of cash flows; amounts in £.</t>
+          <t>Afin Bank Limited (All Africa Capital Limited pre-October 2024) audited/unaudited statement of cash flows; amounts in £. FY2021 NOT DISCLOSED (small-companies exemption - see source note).</t>
         </is>
       </c>
     </row>
@@ -3607,6 +4934,21 @@
           <t>FY2024 (£)</t>
         </is>
       </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>FY2023 (£)</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>FY2022 (£)</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FY2021 (£)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -3615,6 +4957,9 @@
         </is>
       </c>
       <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -3625,167 +4970,294 @@
       <c r="B5" s="6" t="n">
         <v>-5854403</v>
       </c>
+      <c r="C5" s="6" t="n">
+        <v>-1746327</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>-402889</v>
+      </c>
+      <c r="E5" s="6" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Interest received</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="6" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Interest paid</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n">
+        <v>-1263</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="6" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Net cash outflow from operating activities</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B8" s="5" t="n">
         <v>-5854403</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="C8" s="5" t="n">
+        <v>-1747582</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>-402889</v>
+      </c>
+      <c r="E8" s="5" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Investing activities</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Purchase of intangible assets</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>-2668378</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Purchase of property, plant and equipment</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>-52008</v>
-      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Purchase of investments</t>
+          <t>Purchase of intangible assets</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>-9700415</v>
-      </c>
+        <v>-2668378</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>-12000</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
+          <t>Purchase of property, plant and equipment</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>-52008</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>-19717</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Purchase of investments</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>-9700415</v>
+      </c>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
           <t>Finance income</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n">
+      <c r="B13" s="6" t="n">
         <v>75152</v>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Net cash used in investing activities</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B14" s="5" t="n">
         <v>-12345649</v>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="C14" s="5" t="n">
+        <v>-31717</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="5" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Financing activities</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Proceeds from issue of shares</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="n">
-        <v>20523855</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Payment of lease liabilities</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="n">
-        <v>-134783</v>
-      </c>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
+          <t>Proceeds from issue of shares</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>20523855</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>2767153</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>323904</v>
+      </c>
+      <c r="E16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Payment of lease liabilities</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>-134783</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>-23509</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="6" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
           <t>Finance cost</t>
         </is>
       </c>
-      <c r="B16" s="6" t="n">
+      <c r="B18" s="6" t="n">
         <v>-4777</v>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Net cash generated from financing activities</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B19" s="5" t="n">
         <v>20384295</v>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Net increase in cash and cash equivalents</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="n">
-        <v>2184243</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Cash and cash equivalents at the beginning of the year</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="n">
-        <v>971678</v>
-      </c>
+      <c r="C19" s="5" t="n">
+        <v>2743644</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>323904</v>
+      </c>
+      <c r="E19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
+          <t>Net increase in cash and cash equivalents</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>2184243</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>964345</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>-78985</v>
+      </c>
+      <c r="E20" s="5" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Cash and cash equivalents at the beginning of the year</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n">
+        <v>971678</v>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>7333</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>86318</v>
+      </c>
+      <c r="E21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
           <t>Cash and cash equivalents at the end of the year</t>
         </is>
       </c>
-      <c r="B20" s="5" t="n">
+      <c r="B22" s="5" t="n">
         <v>3155921</v>
       </c>
-    </row>
-    <row r="22" ht="165" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>Sources - Afin Bank Limited audited annual report and financial statements for the year ended 31 December 2024:
-FY2024: Statement of cash flows, printed p. 36 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-Ltd-Year-End-Accounts-FV24-FINAL-SIGNED.pdf
-Companies House 2024 accounts filing (filed 29 September 2025) - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history/MzQ4MjgwOTc2M2FkaXF6a2N4/document?download=0&amp;format=pdf
+      <c r="C22" s="5" t="n">
+        <v>971678</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>7333</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>86318</v>
+      </c>
+    </row>
+    <row r="24" ht="225" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Sources - FY2024: Afin Bank Limited audited annual report and financial statements for the year ended 31 December 2024, statement of cash flows, printed p. 36 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-Ltd-Year-End-Accounts-FV24-FINAL-SIGNED.pdf
+FY2023: All Africa Capital Limited audited annual report and financial statements for the year ended 31 December 2023, statement of cash flows, p. 9 (2023 column; 2022 comparative column, itself unaudited per the auditor's report on p. 4) - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history/MzQyNDA1MjMwOGFkaXF6a2N4/document?format=pdf&amp;download=0
+FY2022: as above (FY2023 report's own 2022 comparative column - the standalone FY2022 filing is a balance-sheet-only unaudited filing with no cash flow statement) - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history/MzM5MzI3MzYzNmFkaXF6a2N4/document?format=pdf&amp;download=0
+FY2021: NOT DISCLOSED - All Africa Capital Limited's first accounts (period ended 31 December 2021) take the small companies' exemption from preparing a cash flow statement (FRS 102 Section 1A); no cash flow statement exists for this period in any source reviewed - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history/MzM2MjY4Mzc2MGFkaXF6a2N4/document?format=pdf&amp;download=0
 Companies House filing history - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
+STRUCTURAL NOTE: FY2023/FY2022 route net interest through two new 'Interest received'/'Interest paid' rows under Operating activities (per those years' own statement); FY2024 instead reports 'Finance income' under Investing and 'Finance cost' under Financing (per that year's own statement) - both are reproduced exactly as each year's own source presents them, not forced into a single common layout.
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was incorporated 18 December 2020 as All Africa Capital Limited, traded under that name through FY2021-FY2023, and changed its name to Afin Bank Limited after receiving banking authorisation with restrictions in October 2024. FY2021-FY2023 figures below are therefore All Africa Capital Limited's own pre-bank statutory accounts for the same continuous legal entity, sourced from Companies House (not from afinbank.com, which only hosts the FY2024 bank-era documents).
+FY2020 SELF-SKIPPED IN FULL: the company was incorporated 18 December 2020, so no financial year beginning 1 January 2020 exists for this entity, and no such period was ever filed at Companies House. Its first statutory accounts (filed 16 December 2022) cover the period from incorporation (18 December 2020) to 31 December 2021 - a single ~13.5-month first accounting period, not a discrete FY2020 followed by a discrete FY2021. This was confirmed by reading the full Companies House filing history for company 13090556 (all 4 pages, back to incorporation), not assumed from the entity-creation-date signal alone - https://find-and-update.company-information.service.gov.uk/company/13090556/filing-history</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A24:E24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3797,11 +5269,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3829,33 +5304,64 @@
           <t>FY2024 (£)</t>
         </is>
       </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>FY2023 (£)</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>FY2022 (£)</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FY2021 (£)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
+          <t>Not publicly disclosed / Not applicable</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
           <t>Not publicly disclosed</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Not publicly disclosed</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="150" customHeight="1">
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="180" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Sources - Afin Bank Limited 2024 Annual Report and Pillar 3 Disclosures:
 https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-Ltd-Year-End-Accounts-FV24-FINAL-SIGNED.pdf
 https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.
-NOT DISCLOSED: Afin Bank's balance sheet has no lending product line (assets are Cash, Treasury assets, Receivables, Prepayments, PP&amp;E and intangibles only) and neither the 2024 Annual Report nor the 2024 Pillar 3 disclosure (a small non-complex institution under CRR Article 433b) contains a loan book / IFRS 9 stage / credit risk exposure breakdown.</t>
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was incorporated 18 December 2020 as All Africa Capital Limited, traded under that name through FY2021-FY2023, and changed its name to Afin Bank Limited after receiving banking authorisation with restrictions in October 2024. FY2021-FY2023 figures below are therefore All Africa Capital Limited's own pre-bank statutory accounts for the same continuous legal entity, sourced from Companies House (not from afinbank.com, which only hosts the FY2024 bank-era documents).
+NOT DISCLOSED (FY2024): Afin Bank's balance sheet has no lending product line (assets are Cash, Treasury assets, Receivables, Prepayments, PP&amp;E and intangibles only) and neither the 2024 Annual Report nor the 2024 Pillar 3 disclosure (a small non-complex institution under CRR Article 433b) contains a loan book / IFRS 9 stage / credit risk exposure breakdown.
+NOT APPLICABLE for FY2021-FY2023: All Africa Capital Limited (this entity's name before October 2024) was not a PRA-authorised bank during FY2021-FY2023 and had no Pillar 3 disclosure obligation - its own filed accounts for those years contain no capital/liquidity/leverage/RWA figures of any kind. This is a genuine 'not applicable' (no obligation existed), distinct from 'not publicly disclosed' (an obligated but unpublished figure), which is how FY2024's own non-disclosures are marked.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A6:E6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3867,11 +5373,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3899,6 +5408,21 @@
           <t>FY2024</t>
         </is>
       </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -3909,20 +5433,36 @@
       <c r="B4" s="6" t="n">
         <v>12922</v>
       </c>
-    </row>
-    <row r="6" ht="145" customHeight="1">
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="180" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
 FY2024: UK KM1 Key Metrics, printed pp. 4-5, and UK OV1, printed p. 5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
 Afin Bank annual reports and disclosures page - https://afinbank.com/about/annual-reports-and-disclosures/
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was incorporated 18 December 2020 as All Africa Capital Limited, traded under that name through FY2021-FY2023, and changed its name to Afin Bank Limited after receiving banking authorisation with restrictions in October 2024. FY2021-FY2023 figures below are therefore All Africa Capital Limited's own pre-bank statutory accounts for the same continuous legal entity, sourced from Companies House (not from afinbank.com, which only hosts the FY2024 bank-era documents).
+NOT APPLICABLE for FY2021-FY2023: All Africa Capital Limited (this entity's name before October 2024) was not a PRA-authorised bank during FY2021-FY2023 and had no Pillar 3 disclosure obligation - its own filed accounts for those years contain no capital/liquidity/leverage/RWA figures of any kind. This is a genuine 'not applicable' (no obligation existed), distinct from 'not publicly disclosed' (an obligated but unpublished figure), which is how FY2024's own non-disclosures are marked.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A6:E6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3934,11 +5474,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3966,6 +5509,21 @@
           <t>FY2024</t>
         </is>
       </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -3978,20 +5536,36 @@
           <t>418.5%</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="145" customHeight="1">
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="180" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
 FY2024: UK KM1 Key Metrics, printed pp. 4-5, and UK OV1, printed p. 5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
 Afin Bank annual reports and disclosures page - https://afinbank.com/about/annual-reports-and-disclosures/
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was incorporated 18 December 2020 as All Africa Capital Limited, traded under that name through FY2021-FY2023, and changed its name to Afin Bank Limited after receiving banking authorisation with restrictions in October 2024. FY2021-FY2023 figures below are therefore All Africa Capital Limited's own pre-bank statutory accounts for the same continuous legal entity, sourced from Companies House (not from afinbank.com, which only hosts the FY2024 bank-era documents).
+NOT APPLICABLE for FY2021-FY2023: All Africa Capital Limited (this entity's name before October 2024) was not a PRA-authorised bank during FY2021-FY2023 and had no Pillar 3 disclosure obligation - its own filed accounts for those years contain no capital/liquidity/leverage/RWA figures of any kind. This is a genuine 'not applicable' (no obligation existed), distinct from 'not publicly disclosed' (an obligated but unpublished figure), which is how FY2024's own non-disclosures are marked.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A6:E6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4003,11 +5577,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4035,6 +5612,21 @@
           <t>FY2024</t>
         </is>
       </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -4045,20 +5637,36 @@
       <c r="B4" s="6" t="n">
         <v>12922</v>
       </c>
-    </row>
-    <row r="6" ht="145" customHeight="1">
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="180" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Sources - Afin Bank Limited standalone Pillar 3 Disclosures for the year ended 31 December 2024:
 FY2024: UK KM1 Key Metrics, printed pp. 4-5, and UK OV1, printed p. 5 - https://afinbank.com/wp-content/uploads/2025/09/Afin-Bank-2024-Pillar-3-Disclosures-FINAL.pdf
 Afin Bank annual reports and disclosures page - https://afinbank.com/about/annual-reports-and-disclosures/
-ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was formerly named All Africa Capital Limited and changed its name after receiving banking authorisation with restrictions in October 2024.</t>
+ENTITY NOTE: Afin Bank Limited (company 13090556, FRN 1004742) is the UK legal entity covered here. The 2024 Pillar 3 report says the disclosure scope applies to Afin Bank Limited only; it is a majority-owned subsidiary of WAICA Reinsurance Corporation PLC, but no parent-level figures are substituted. The company was incorporated 18 December 2020 as All Africa Capital Limited, traded under that name through FY2021-FY2023, and changed its name to Afin Bank Limited after receiving banking authorisation with restrictions in October 2024. FY2021-FY2023 figures below are therefore All Africa Capital Limited's own pre-bank statutory accounts for the same continuous legal entity, sourced from Companies House (not from afinbank.com, which only hosts the FY2024 bank-era documents).
+NOT APPLICABLE for FY2021-FY2023: All Africa Capital Limited (this entity's name before October 2024) was not a PRA-authorised bank during FY2021-FY2023 and had no Pillar 3 disclosure obligation - its own filed accounts for those years contain no capital/liquidity/leverage/RWA figures of any kind. This is a genuine 'not applicable' (no obligation existed), distinct from 'not publicly disclosed' (an obligated but unpublished figure), which is how FY2024's own non-disclosures are marked.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A6:E6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>